<commit_message>
Type 01: mitred corners + reveal slips on the wall coursing, editable BOQ + Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/T01/downloads/DG-T01 Turnkey BOQ.xlsx
+++ b/T01/downloads/DG-T01 Turnkey BOQ.xlsx
@@ -2358,7 +2358,7 @@
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3270,7 +3270,7 @@
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>

</xml_diff>